<commit_message>
Add project README.md and update raw Excel source data
</commit_message>
<xml_diff>
--- a/reference/Idle Apocalypse Nether Raw Data.xlsx
+++ b/reference/Idle Apocalypse Nether Raw Data.xlsx
@@ -1,14 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/243a7b8946868a62/Documents/Coding Projects/Idle Apocalypse Nether Costs/reference/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_4432978DB50C4271B1C2ECC3F609CF911F46E402" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33D4EF1F-23D5-4D95-BFCB-3218F94E4CAF}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Targets" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Nether Creatures" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Variable Upgrades" sheetId="3" r:id="rId7"/>
+    <sheet name="Targets" sheetId="1" r:id="rId1"/>
+    <sheet name="Nether Creatures" sheetId="2" r:id="rId2"/>
+    <sheet name="Variable Upgrades" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -216,18 +225,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="m-d"/>
+    <numFmt numFmtId="164" formatCode="m\-d"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -238,51 +248,44 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -472,17 +475,20 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:G37"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -505,7 +511,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -513,13 +519,13 @@
         <v>8</v>
       </c>
       <c r="C2" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="G2" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -527,13 +533,13 @@
         <v>8</v>
       </c>
       <c r="C3" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E3" s="1">
-        <v>10.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -541,16 +547,16 @@
         <v>8</v>
       </c>
       <c r="C4" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="D4" s="1">
-        <v>60.0</v>
+        <v>60</v>
       </c>
       <c r="F4" s="1">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -558,16 +564,16 @@
         <v>9</v>
       </c>
       <c r="C5" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D5" s="1">
-        <v>40.0</v>
+        <v>40</v>
       </c>
       <c r="G5" s="1">
-        <v>10.0</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -575,13 +581,13 @@
         <v>9</v>
       </c>
       <c r="C6" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F6" s="1">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -589,16 +595,16 @@
         <v>9</v>
       </c>
       <c r="C7" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E7" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="F7" s="1">
-        <v>6.0</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -606,16 +612,16 @@
         <v>10</v>
       </c>
       <c r="C8" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="G8" s="1">
-        <v>15.0</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -623,16 +629,16 @@
         <v>10</v>
       </c>
       <c r="C9" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="D9" s="1">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="E9" s="1">
-        <v>20.0</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -640,10 +646,10 @@
         <v>12</v>
       </c>
       <c r="E10" s="1">
-        <v>15.0</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -651,13 +657,13 @@
         <v>13</v>
       </c>
       <c r="D11" s="1">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="E11" s="1">
-        <v>10.0</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
@@ -665,13 +671,13 @@
         <v>14</v>
       </c>
       <c r="D12" s="1">
-        <v>75.0</v>
+        <v>75</v>
       </c>
       <c r="E12" s="1">
-        <v>15.0</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -679,10 +685,10 @@
         <v>15</v>
       </c>
       <c r="D13" s="1">
-        <v>50.0</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>11</v>
       </c>
@@ -690,13 +696,13 @@
         <v>16</v>
       </c>
       <c r="E14" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="F14" s="1">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>11</v>
       </c>
@@ -704,10 +710,10 @@
         <v>17</v>
       </c>
       <c r="D15" s="1">
-        <v>75.0</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>11</v>
       </c>
@@ -715,10 +721,10 @@
         <v>18</v>
       </c>
       <c r="F16" s="1">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
@@ -726,13 +732,13 @@
         <v>19</v>
       </c>
       <c r="D17" s="1">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="F17" s="1">
-        <v>6.0</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>11</v>
       </c>
@@ -740,10 +746,10 @@
         <v>20</v>
       </c>
       <c r="D18" s="1">
-        <v>25.0</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>11</v>
       </c>
@@ -751,13 +757,13 @@
         <v>21</v>
       </c>
       <c r="D19" s="1">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="E19" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>11</v>
       </c>
@@ -765,13 +771,13 @@
         <v>22</v>
       </c>
       <c r="E20" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="F20" s="1">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>11</v>
       </c>
@@ -779,10 +785,10 @@
         <v>23</v>
       </c>
       <c r="D21" s="1">
-        <v>35.0</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>11</v>
       </c>
@@ -790,52 +796,52 @@
         <v>24</v>
       </c>
       <c r="D22" s="1">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="E22" s="1">
-        <v>10.0</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C23" s="1">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="D23" s="1">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="E23" s="1">
-        <v>25.0</v>
-      </c>
-    </row>
-    <row r="24">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C24" s="1">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="E24" s="1">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="F24" s="1">
-        <v>25.0</v>
-      </c>
-    </row>
-    <row r="25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C25" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="F25" s="1">
-        <v>50.0</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>26</v>
       </c>
@@ -844,10 +850,10 @@
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="1">
-        <v>100.0</v>
-      </c>
-    </row>
-    <row r="27">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>26</v>
       </c>
@@ -856,10 +862,10 @@
       </c>
       <c r="C27" s="2"/>
       <c r="E27" s="1">
-        <v>25.0</v>
-      </c>
-    </row>
-    <row r="28">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -868,10 +874,10 @@
       </c>
       <c r="C28" s="2"/>
       <c r="F28" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="29">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>26</v>
       </c>
@@ -879,10 +885,10 @@
         <v>30</v>
       </c>
       <c r="D29" s="1">
-        <v>200.0</v>
-      </c>
-    </row>
-    <row r="30">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>26</v>
       </c>
@@ -890,10 +896,10 @@
         <v>31</v>
       </c>
       <c r="E30" s="1">
-        <v>50.0</v>
-      </c>
-    </row>
-    <row r="31">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>26</v>
       </c>
@@ -901,10 +907,10 @@
         <v>32</v>
       </c>
       <c r="F31" s="1">
-        <v>10.0</v>
-      </c>
-    </row>
-    <row r="32">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>26</v>
       </c>
@@ -912,10 +918,10 @@
         <v>33</v>
       </c>
       <c r="D32" s="1">
-        <v>300.0</v>
-      </c>
-    </row>
-    <row r="33">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>26</v>
       </c>
@@ -923,10 +929,10 @@
         <v>34</v>
       </c>
       <c r="E33" s="1">
-        <v>75.0</v>
-      </c>
-    </row>
-    <row r="34">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>26</v>
       </c>
@@ -934,10 +940,10 @@
         <v>35</v>
       </c>
       <c r="F34" s="1">
-        <v>25.0</v>
-      </c>
-    </row>
-    <row r="35">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>26</v>
       </c>
@@ -945,10 +951,10 @@
         <v>36</v>
       </c>
       <c r="D35" s="1">
-        <v>500.0</v>
-      </c>
-    </row>
-    <row r="36">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>26</v>
       </c>
@@ -956,10 +962,10 @@
         <v>37</v>
       </c>
       <c r="E36" s="1">
-        <v>100.0</v>
-      </c>
-    </row>
-    <row r="37">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>26</v>
       </c>
@@ -967,22 +973,23 @@
         <v>38</v>
       </c>
       <c r="F37" s="1">
-        <v>50.0</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>39</v>
       </c>
@@ -1014,91 +1021,91 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D2" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="E2" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>49</v>
       </c>
       <c r="G2" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="H2" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="I2" s="1">
-        <v>7.0</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="C3" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="E3" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>50</v>
       </c>
       <c r="G3" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="H3" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="I3" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B4" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C4" s="1">
-        <v>12.0</v>
+        <v>0</v>
       </c>
       <c r="D4" s="1">
-        <v>0.0</v>
+        <v>12</v>
       </c>
       <c r="E4" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>53</v>
       </c>
       <c r="G4" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>54</v>
@@ -1108,21 +1115,22 @@
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="47.5"/>
+    <col min="2" max="2" width="47.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1139,7 +1147,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>60</v>
       </c>
@@ -1147,16 +1155,16 @@
         <v>61</v>
       </c>
       <c r="C2" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D2" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>63</v>
       </c>
@@ -1168,6 +1176,6 @@
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>